<commit_message>
feat: add controlled petrochemical catalog importer
</commit_message>
<xml_diff>
--- a/outputs/smartkey-products-2026-07-21/smartkey-petrochemical-catalog.xlsx
+++ b/outputs/smartkey-products-2026-07-21/smartkey-petrochemical-catalog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8d2c9a809e4845c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="R120ff28d26674035"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical Properties" sheetId="3" r:id="R9770546cc4a84c6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="R1f672bfcf6b34124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8b14fe071175462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="R4c6a9a7c5a4d49ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical Properties" sheetId="3" r:id="R09c88bd7a7b64d56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="R94da5aaaa9924669"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,7 +485,7 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>Descriptions are original SmartKey summaries generated from product names, categories and applications. Technical values remain linked to their source page. Source images are not cleared for publication and are marked Pending written permission. Every product remains subject to supplier confirmation before publication or quotation.</x:v>
+        <x:v>Descriptions are original SmartKey summaries generated from product names, categories and applications. Technical values remain linked to their source page. The owner confirmed authorization to republish the source catalog and images on 2026-07-21. SmartKey is an authorized sales representative, not the manufacturer; current specifications and commercial terms remain subject to inquiry confirmation.</x:v>
       </x:c>
       <x:c r="F5" s="17"/>
       <x:c r="G5" s="17"/>
@@ -827,7 +827,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/ABS.webp</x:v>
       </x:c>
       <x:c r="H2" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I2" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hr-2320</x:v>
@@ -848,7 +848,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O2" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -874,7 +874,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/ABS.webp</x:v>
       </x:c>
       <x:c r="H3" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I3" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hr-2340</x:v>
@@ -895,7 +895,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O3" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -921,7 +921,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/ABS.webp</x:v>
       </x:c>
       <x:c r="H4" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I4" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-sd-0150</x:v>
@@ -942,7 +942,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O4" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -968,7 +968,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/ABS.webp</x:v>
       </x:c>
       <x:c r="H5" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I5" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-sv-0157</x:v>
@@ -989,7 +989,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O5" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1013,7 +1013,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/METHANOL.webp</x:v>
       </x:c>
       <x:c r="H6" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I6" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=methanol</x:v>
@@ -1034,7 +1034,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O6" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1060,7 +1060,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/EPS.jpg</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I7" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-eps</x:v>
@@ -1081,7 +1081,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O7" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1107,7 +1107,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/GPPS.jpg</x:v>
       </x:c>
       <x:c r="H8" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I8" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-gpps-1160</x:v>
@@ -1128,7 +1128,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O8" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1154,7 +1154,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/GPPS.jpg</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I9" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-gpps-1460</x:v>
@@ -1175,7 +1175,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O9" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1201,7 +1201,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/GPPS.jpg</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I10" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-gpps-1540</x:v>
@@ -1222,7 +1222,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O10" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1248,7 +1248,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/DEG.webp</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I11" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=deg-diethylene-glycol</x:v>
@@ -1269,7 +1269,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O11" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1295,7 +1295,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/Paraffin-wax3-5.jpg</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I12" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=lemon-petroleum-jelly</x:v>
@@ -1316,7 +1316,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O12" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1342,7 +1342,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/MEG.webp</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=monoethylene-glycol-meg</x:v>
@@ -1363,7 +1363,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O13" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1389,7 +1389,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/Paraffin-Wax-1-3.webp</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I14" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=paraffin-wax1-3</x:v>
@@ -1410,7 +1410,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O14" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1436,7 +1436,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/Paraffin-wax3-5.jpg</x:v>
       </x:c>
       <x:c r="H15" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I15" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=paraffin-wax3-5</x:v>
@@ -1457,7 +1457,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O15" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1483,7 +1483,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/Paraffin-wax3-5.jpg</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I16" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=paraffin-wax5-8</x:v>
@@ -1504,7 +1504,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O16" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1530,7 +1530,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/Paraffin-wax3-5.jpg</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=paraffin-wax%e2%89%a42</x:v>
@@ -1551,7 +1551,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O17" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1577,7 +1577,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/PETROLEUM-JELLY.webp</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=petroleum-jelly</x:v>
@@ -1598,7 +1598,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O18" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1624,7 +1624,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/TEG.webp</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=teg-triethylene-glycol</x:v>
@@ -1645,7 +1645,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O19" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1671,7 +1671,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/Ultra-Snow-White-petroleum-jelly.webp</x:v>
       </x:c>
       <x:c r="H20" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ultra-snow-white-petroleum-jelly</x:v>
@@ -1692,7 +1692,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O20" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1718,7 +1718,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/Paraffin-wax3-5.jpg</x:v>
       </x:c>
       <x:c r="H21" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I21" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=white-petroleum-jelly</x:v>
@@ -1739,7 +1739,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O21" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1765,7 +1765,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H22" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I22" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-7750</x:v>
@@ -1786,7 +1786,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O22" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1812,7 +1812,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H23" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I23" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-gd107255</x:v>
@@ -1833,7 +1833,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O23" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1859,7 +1859,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/A104750.webp</x:v>
       </x:c>
       <x:c r="H24" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I24" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a104750</x:v>
@@ -1880,7 +1880,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O24" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1906,7 +1906,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H25" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a104760</x:v>
@@ -1927,7 +1927,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O25" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1953,7 +1953,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H26" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a105010-t2n</x:v>
@@ -1974,7 +1974,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O26" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2000,7 +2000,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H27" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a106255</x:v>
@@ -2021,7 +2021,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O27" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2047,7 +2047,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H28" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I28" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a107250</x:v>
@@ -2068,7 +2068,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O28" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2094,7 +2094,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H29" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a107255</x:v>
@@ -2115,7 +2115,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O29" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2141,7 +2141,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H30" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a107260</x:v>
@@ -2162,7 +2162,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O30" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2188,7 +2188,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H31" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-7740f2</x:v>
@@ -2209,7 +2209,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O31" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2235,7 +2235,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H32" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a107745</x:v>
@@ -2256,7 +2256,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O32" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2282,7 +2282,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H33" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a107746</x:v>
@@ -2303,7 +2303,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O33" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2329,7 +2329,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H34" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I34" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a108255</x:v>
@@ -2350,7 +2350,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O34" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2376,7 +2376,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H35" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a9450f</x:v>
@@ -2397,7 +2397,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O35" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2423,7 +2423,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H36" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I36" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a9455f</x:v>
@@ -2444,7 +2444,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O36" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2470,7 +2470,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE.webp</x:v>
       </x:c>
       <x:c r="H37" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=agc107260</x:v>
@@ -2491,7 +2491,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O37" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2517,7 +2517,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE1080.webp</x:v>
       </x:c>
       <x:c r="H38" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I38" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=hdpe-1080</x:v>
@@ -2538,7 +2538,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O38" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2564,7 +2564,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE-S104261A-1.webp</x:v>
       </x:c>
       <x:c r="H39" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I39" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=hdpe-s104261a</x:v>
@@ -2585,7 +2585,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O39" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2611,7 +2611,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE-S4265-1.webp</x:v>
       </x:c>
       <x:c r="H40" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I40" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=hbm-4265</x:v>
@@ -2632,7 +2632,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O40" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2658,7 +2658,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE-S5020.webp</x:v>
       </x:c>
       <x:c r="H41" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I41" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=hdpe-s5020</x:v>
@@ -2679,7 +2679,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O41" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2705,7 +2705,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE-S5110.webp</x:v>
       </x:c>
       <x:c r="H42" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I42" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=hdpe-s5110</x:v>
@@ -2726,7 +2726,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O42" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2752,7 +2752,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE-S5510.webp</x:v>
       </x:c>
       <x:c r="H43" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I43" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=hdpe-s5510</x:v>
@@ -2773,7 +2773,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O43" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2799,7 +2799,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/HDPE-SPE80.webp</x:v>
       </x:c>
       <x:c r="H44" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I44" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=hdpe-spe80</x:v>
@@ -2820,7 +2820,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O44" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2846,7 +2846,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H45" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I45" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ilhd-107000f</x:v>
@@ -2867,7 +2867,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O45" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -2893,7 +2893,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H46" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I46" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=j-104760-bl3</x:v>
@@ -2914,7 +2914,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O46" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2940,7 +2940,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H47" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I47" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=j-1060507-uv</x:v>
@@ -2961,7 +2961,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O47" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2987,7 +2987,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H48" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I48" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=j-109450f-ex5</x:v>
@@ -3008,7 +3008,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O48" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -3034,7 +3034,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H49" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I49" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=j-10crp100-black</x:v>
@@ -3055,7 +3055,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O49" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -3081,7 +3081,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H50" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I50" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=j-10crp100-n-pe100</x:v>
@@ -3102,7 +3102,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O50" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -3128,7 +3128,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H51" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I51" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=j-hd-105000-s</x:v>
@@ -3149,7 +3149,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O51" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -3175,7 +3175,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H52" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I52" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=jhd-1052505-uv</x:v>
@@ -3196,7 +3196,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O52" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -3222,7 +3222,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H53" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I53" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=jhd-1052518</x:v>
@@ -3243,7 +3243,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O53" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3269,7 +3269,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H54" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I54" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hd-103840-ua</x:v>
@@ -3290,7 +3290,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O54" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3316,7 +3316,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H55" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I55" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hd-104005-ea</x:v>
@@ -3337,7 +3337,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O55" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3363,7 +3363,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H56" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I56" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hd-104440-ea</x:v>
@@ -3384,7 +3384,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O56" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -3410,7 +3410,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H57" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I57" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hd-105030-sa</x:v>
@@ -3431,7 +3431,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O57" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3457,7 +3457,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H58" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I58" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hd-105218-ua</x:v>
@@ -3478,7 +3478,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O58" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -3504,7 +3504,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H59" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I59" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hd-106040-ua</x:v>
@@ -3525,7 +3525,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O59" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -3551,7 +3551,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H60" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I60" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hd-106070-ua</x:v>
@@ -3572,7 +3572,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O60" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -3598,7 +3598,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HIPS-Polystyrene.jpg</x:v>
       </x:c>
       <x:c r="H61" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I61" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hips-7240</x:v>
@@ -3619,7 +3619,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O61" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -3645,7 +3645,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HIPS-Polystyrene.jpg</x:v>
       </x:c>
       <x:c r="H62" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I62" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hips-7350escr</x:v>
@@ -3666,7 +3666,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O62" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -3692,7 +3692,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/HIPS-Polystyrene.jpg</x:v>
       </x:c>
       <x:c r="H63" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I63" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-hips-8350</x:v>
@@ -3713,7 +3713,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O63" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3739,7 +3739,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H64" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I64" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-202420d</x:v>
@@ -3760,7 +3760,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O64" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3786,7 +3786,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H65" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I65" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-202420f</x:v>
@@ -3807,7 +3807,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O65" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3833,7 +3833,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H66" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I66" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-202420h</x:v>
@@ -3854,7 +3854,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O66" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3880,7 +3880,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H67" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I67" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-202426f</x:v>
@@ -3901,7 +3901,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O67" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3927,7 +3927,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H68" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I68" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=305</x:v>
@@ -3948,7 +3948,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O68" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -3974,7 +3974,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H69" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I69" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-203020h</x:v>
@@ -3995,7 +3995,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O69" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -4021,7 +4021,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H70" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I70" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-203020k</x:v>
@@ -4042,7 +4042,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O70" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -4068,7 +4068,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H71" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I71" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-203026h</x:v>
@@ -4089,7 +4089,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O71" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -4115,7 +4115,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE.webp</x:v>
       </x:c>
       <x:c r="H72" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I72" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a201800s</x:v>
@@ -4136,7 +4136,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O72" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -4162,7 +4162,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE-S201969.webp</x:v>
       </x:c>
       <x:c r="H73" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I73" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ldpe-s201969</x:v>
@@ -4183,7 +4183,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O73" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -4209,7 +4209,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE-S202047A.webp</x:v>
       </x:c>
       <x:c r="H74" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I74" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ldpe-s202047a</x:v>
@@ -4230,7 +4230,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O74" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -4256,7 +4256,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE-S202119.webp</x:v>
       </x:c>
       <x:c r="H75" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I75" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ldpe-s202119</x:v>
@@ -4277,7 +4277,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O75" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -4303,7 +4303,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE-S202125A.webp</x:v>
       </x:c>
       <x:c r="H76" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I76" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ldpe-s202125a</x:v>
@@ -4324,7 +4324,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O76" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -4350,7 +4350,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE-S202130.webp</x:v>
       </x:c>
       <x:c r="H77" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I77" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ldpe-s202130</x:v>
@@ -4371,7 +4371,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O77" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -4397,7 +4397,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE-S202185.webp</x:v>
       </x:c>
       <x:c r="H78" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I78" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ldpe-s202185</x:v>
@@ -4418,7 +4418,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O78" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -4444,7 +4444,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LDPE-S202575.webp</x:v>
       </x:c>
       <x:c r="H79" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I79" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=ldpe-s202575</x:v>
@@ -4465,7 +4465,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O79" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -4491,7 +4491,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LLDPE.webp</x:v>
       </x:c>
       <x:c r="H80" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I80" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-30205aa</x:v>
@@ -4512,7 +4512,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O80" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -4538,7 +4538,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LLDPE.webp</x:v>
       </x:c>
       <x:c r="H81" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I81" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-30209aa</x:v>
@@ -4559,7 +4559,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O81" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -4585,7 +4585,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LLDPE.webp</x:v>
       </x:c>
       <x:c r="H82" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I82" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-30209kj</x:v>
@@ -4606,7 +4606,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O82" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -4632,7 +4632,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LLDPE.webp</x:v>
       </x:c>
       <x:c r="H83" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I83" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-30220aa</x:v>
@@ -4653,7 +4653,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O83" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -4679,7 +4679,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/LLDPE.webp</x:v>
       </x:c>
       <x:c r="H84" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I84" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=a-30220kj</x:v>
@@ -4700,7 +4700,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O84" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -4726,7 +4726,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/LLDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H85" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I85" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=j-ll-30235f6</x:v>
@@ -4747,7 +4747,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O85" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -4773,7 +4773,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/LLDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H86" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I86" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-ll-300209-aa</x:v>
@@ -4794,7 +4794,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O86" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -4820,7 +4820,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/LLDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H87" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I87" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-ll-300209-kj</x:v>
@@ -4841,7 +4841,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O87" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -4867,7 +4867,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/LLDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H88" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I88" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-ll-300220-aa</x:v>
@@ -4888,7 +4888,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O88" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4914,7 +4914,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/LLDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H89" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I89" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-ll-300220-kj</x:v>
@@ -4935,7 +4935,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O89" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4961,7 +4961,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/LLDPE-2.jpg</x:v>
       </x:c>
       <x:c r="H90" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I90" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-ll-304110-aa</x:v>
@@ -4982,7 +4982,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O90" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -5008,7 +5008,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/MDPE-S403313.webp</x:v>
       </x:c>
       <x:c r="H91" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I91" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=mdpe-s403313</x:v>
@@ -5029,7 +5029,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O91" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -5055,7 +5055,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/10/MDPE-S403820.webp</x:v>
       </x:c>
       <x:c r="H92" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I92" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=mdpe-s403820</x:v>
@@ -5076,7 +5076,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O92" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -5100,7 +5100,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/Base-oils.jpeg</x:v>
       </x:c>
       <x:c r="H93" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I93" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=base-oil-sn-150</x:v>
@@ -5121,7 +5121,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O93" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -5145,7 +5145,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/Base-oils.jpeg</x:v>
       </x:c>
       <x:c r="H94" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I94" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=base-oil-sn-350</x:v>
@@ -5166,7 +5166,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O94" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -5190,7 +5190,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/Base-oils.jpeg</x:v>
       </x:c>
       <x:c r="H95" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I95" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=base-oil-sn-50</x:v>
@@ -5211,7 +5211,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O95" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -5235,7 +5235,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/Bitumen.jpg</x:v>
       </x:c>
       <x:c r="H96" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I96" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=bitumen</x:v>
@@ -5256,7 +5256,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O96" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -5280,7 +5280,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/PP.webp</x:v>
       </x:c>
       <x:c r="H97" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I97" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-pph-hd-225</x:v>
@@ -5301,7 +5301,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O97" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -5327,7 +5327,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/PP.webp</x:v>
       </x:c>
       <x:c r="H98" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I98" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-pph-xd-045</x:v>
@@ -5348,7 +5348,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O98" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -5372,7 +5372,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/PP.webp</x:v>
       </x:c>
       <x:c r="H99" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I99" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=t-pph-yd-225</x:v>
@@ -5393,7 +5393,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O99" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -5417,7 +5417,7 @@
         <x:v>https://chemportal.com.tr/wp-content/uploads/2024/11/Urea46.png</x:v>
       </x:c>
       <x:c r="H100" s="24" t="str">
-        <x:v>Pending written permission</x:v>
+        <x:v>Authorized — owner confirmed 2026-07-21</x:v>
       </x:c>
       <x:c r="I100" s="24" t="str">
         <x:v>https://chemportal.com.tr/?product=granule-urea-46</x:v>
@@ -5438,7 +5438,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O100" s="24" t="str">
-        <x:v>SmartKey Turkey facilitates sourcing and coordination; specifications, availability, pricing and final terms are confirmed by the relevant supplier.</x:v>
+        <x:v>SmartKey Turkey acts as an authorized sales representative and sourcing coordinator; it is not the manufacturer. Current specifications, availability, pricing and final commercial terms are confirmed for each inquiry.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5447,7 +5447,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc66c1c91097a43da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38ce604e5b334f02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31646,7 +31646,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05216738ec934aac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2464d27c02b4286"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31688,7 +31688,7 @@
         <x:v>Image Source URL</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>Reference-only URL. Do not publish until written reuse permission or a replacement image is approved.</x:v>
+        <x:v>Owner confirmed authorization for SmartKey to reuse the source catalog images on 2026-07-21.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -31709,10 +31709,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="28" t="str">
-        <x:v>Intermediary Disclosure</x:v>
+        <x:v>Representative Disclosure</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>SmartKey is a sourcing and coordination intermediary, not the manufacturer or stock owner.</x:v>
+        <x:v>SmartKey is an authorized sales representative and sourcing coordinator, not the manufacturer.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>